<commit_message>
3.1.5 Se modifica la redacción del los correos
</commit_message>
<xml_diff>
--- a/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX Documentación de Resultados.xlsx
+++ b/static/plantillas/XXX-XXX-XXX-X-XXX-XXX-XXX Documentación de Resultados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BID-eduardo.hernande\Desktop\extractor\excel_extractor\static\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2927B407-9EE6-40AE-909A-FE20399F886D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB197D11-75CC-4D75-9D11-466A92252FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{54E05A43-795E-4F4C-A5C1-AD3CF9CBA03F}"/>
   </bookViews>
@@ -130,7 +130,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,8 +225,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -242,7 +242,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -259,9 +259,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -299,7 +299,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -405,7 +405,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -547,7 +547,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -556,7 +556,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9472DF1C-DCD0-4BB3-A751-5BF20BDDD3E2}">
   <dimension ref="A2:N31"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="9.26953125" customWidth="1"/>
@@ -570,7 +570,7 @@
     <col min="16" max="16" width="21.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -588,7 +588,7 @@
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14">
       <c r="A3" s="9" t="s">
         <v>1</v>
       </c>
@@ -614,7 +614,7 @@
       </c>
       <c r="N3" s="12"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14">
       <c r="A4" s="9" t="s">
         <v>3</v>
       </c>
@@ -640,7 +640,7 @@
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14">
       <c r="A5" s="9" t="s">
         <v>6</v>
       </c>
@@ -658,7 +658,7 @@
       <c r="M5" s="9"/>
       <c r="N5" s="9"/>
     </row>
-    <row r="6" spans="1:14" ht="135.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="135.75" customHeight="1">
       <c r="A6" s="15"/>
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
@@ -674,7 +674,7 @@
       <c r="M6" s="15"/>
       <c r="N6" s="15"/>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14">
       <c r="A7" s="9" t="s">
         <v>7</v>
       </c>
@@ -692,7 +692,7 @@
       <c r="M7" s="9"/>
       <c r="N7" s="9"/>
     </row>
-    <row r="8" spans="1:14" ht="188.25" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="188.25" customHeight="1">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -708,7 +708,7 @@
       <c r="M8" s="15"/>
       <c r="N8" s="15"/>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14">
       <c r="A9" s="3" t="s">
         <v>11</v>
       </c>
@@ -734,7 +734,7 @@
       </c>
       <c r="N9" s="9"/>
     </row>
-    <row r="10" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="249" customHeight="1">
       <c r="A10" s="6" t="s">
         <v>17</v>
       </c>
@@ -756,7 +756,7 @@
       </c>
       <c r="N10" s="10"/>
     </row>
-    <row r="11" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="249" customHeight="1">
       <c r="A11" s="6" t="s">
         <v>20</v>
       </c>
@@ -778,7 +778,7 @@
       </c>
       <c r="N11" s="10"/>
     </row>
-    <row r="12" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="249" customHeight="1">
       <c r="A12" s="6" t="s">
         <v>21</v>
       </c>
@@ -800,7 +800,7 @@
       </c>
       <c r="N12" s="10"/>
     </row>
-    <row r="13" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="249" customHeight="1">
       <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
@@ -822,7 +822,7 @@
       </c>
       <c r="N13" s="10"/>
     </row>
-    <row r="14" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="249" customHeight="1">
       <c r="A14" s="6" t="s">
         <v>23</v>
       </c>
@@ -844,7 +844,7 @@
       </c>
       <c r="N14" s="10"/>
     </row>
-    <row r="15" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="249" customHeight="1">
       <c r="A15" s="6" t="s">
         <v>24</v>
       </c>
@@ -866,7 +866,7 @@
       </c>
       <c r="N15" s="10"/>
     </row>
-    <row r="16" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="249" customHeight="1">
       <c r="A16" s="6" t="s">
         <v>25</v>
       </c>
@@ -888,7 +888,7 @@
       </c>
       <c r="N16" s="10"/>
     </row>
-    <row r="17" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:14" ht="249" customHeight="1">
       <c r="A17" s="6" t="s">
         <v>26</v>
       </c>
@@ -910,7 +910,7 @@
       </c>
       <c r="N17" s="10"/>
     </row>
-    <row r="18" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:14" ht="249" customHeight="1">
       <c r="A18" s="6" t="s">
         <v>27</v>
       </c>
@@ -932,7 +932,7 @@
       </c>
       <c r="N18" s="10"/>
     </row>
-    <row r="19" spans="1:14" ht="249" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:14" ht="249" customHeight="1">
       <c r="A19" s="6" t="s">
         <v>28</v>
       </c>
@@ -954,25 +954,25 @@
       </c>
       <c r="N19" s="10"/>
     </row>
-    <row r="20" spans="1:14" ht="57" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="9" t="s">
+    <row r="20" spans="1:14" ht="57" customHeight="1">
+      <c r="A20" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+      <c r="N20" s="10"/>
+    </row>
+    <row r="31" spans="1:14">
       <c r="L31" s="7"/>
     </row>
   </sheetData>

</xml_diff>